<commit_message>
Version1.2:relation works but from java, also work from  from python
</commit_message>
<xml_diff>
--- a/uploads/z-Zigeunerpaar.xlsx
+++ b/uploads/z-Zigeunerpaar.xlsx
@@ -164,7 +164,7 @@
     <t xml:space="preserve">nodeType</t>
   </si>
   <si>
-    <t xml:space="preserve">Painitng</t>
+    <t xml:space="preserve">Painting</t>
   </si>
 </sst>
 </file>
@@ -248,24 +248,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -462,12 +458,12 @@
   <dimension ref="A1:B32"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30.38"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -685,10 +681,10 @@
       <c r="B31" s="3"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="3" t="s">
         <v>47</v>
       </c>
     </row>

</xml_diff>